<commit_message>
market radar trying to fix geoapify
</commit_message>
<xml_diff>
--- a/market-radar-settings-reference.xlsx
+++ b/market-radar-settings-reference.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E75"/>
+  <dimension ref="A1:E83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -558,18 +558,18 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Only tried once every Overpass mirror has failed</t>
+          <t>Only tried once every Overpass mirror has failed (or reported a runtime error)</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>GOOGLE_PLACES_API_KEY -- Cloudflare Worker Secret, NOT this sheet</t>
+          <t>GEOAPIFY_API_KEY -- Cloudflare Worker Secret, NOT this sheet</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Free, 3,000 credits/day, no card at myprojects.geoapify.com. NEVER paste the real key into this file -- Settings &gt; Variables and Secrets on the Worker only.</t>
+          <t>Free, 3,000 credits/day, no card at myprojects.geoapify.com. NEVER paste the real key into this file -- Settings &gt; Variables and Secrets on the Worker only. THE SECRET NAME MUST BE EXACTLY GEOAPIFY_API_KEY. CORRECTED 2026-09-20: this row used to say GOOGLE_PLACES_API_KEY (copy-paste error) -- see the 'How to use this' tab.</t>
         </is>
       </c>
     </row>
@@ -1269,7 +1269,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
@@ -1506,7 +1505,6 @@
       </c>
       <c r="E58" s="3" t="inlineStr"/>
     </row>
-    <row r="59"/>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
@@ -1636,7 +1634,6 @@
         </is>
       </c>
     </row>
-    <row r="67"/>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
@@ -1782,6 +1779,155 @@
       <c r="E75" s="3" t="inlineStr">
         <is>
           <t>Large private employers deliberately excluded — no reliable OSM tag exists for this; use the vacancy-style manual notepad if it matters for a specific spot</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>GEOAPIFY BACKSTOP &amp; DIAGNOSTICS -- added 2026-09-20 (v1.4.0)</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="n"/>
+      <c r="C77" s="2" t="n"/>
+      <c r="D77" s="2" t="n"/>
+      <c r="E77" s="2" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>Geoapify max places per backstop call</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="n"/>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>GEOAPIFY_RESULT_LIMIT, market-radar-proxy-worker.js</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>500 is Geoapify's documented maximum and applies to ALL categories combined, returned nearest-first; if the cap is hit the page warns the count may be an undercount (big drive catchments). Billing appears to be about 1 credit per 20 places RETURNED (inferred from Geoapify's own sample repo: 60,000 places/day on the 3,000-credit free budget; the Places pricing section itself could not be read), so a full answer could cost ~25 credits. Lower this to cap spend per backstop call.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>Backstop fire-drill switch</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>Off (variable not set)</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="n"/>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>FORCE_OVERPASS_FAIL -- a VARIABLE (Type: Text) on the Worker (Settings &gt; Variables and Secrets), not a secret</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>Set to 1 to skip Overpass AND its cache, forcing the Geoapify backstop. Run one analysis: the page should say 'via Geoapify backstop'. Then DELETE the variable. Any value other than 1 does nothing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>Overpass soft-failure handling</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>On, always (not adjustable)</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="n"/>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>SOFT-FAILURE CHECK inside fetchOverpassPOIs, market-radar-proxy-worker.js</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>Overpass reports timeouts and out-of-memory as HTTP 200 plus a 'remark' field. A remark containing 'runtime error' (or any remark with zero results) is now treated as a failed mirror: skipped and never cached. A genuine empty answer (no remark) is still accepted as a real '0 competitors'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>Worker version (shown on the page)</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>1.4.0</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="n"/>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>WORKER_VERSION, market-radar-proxy-worker.js</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="inlineStr">
+        <is>
+          <t>The page prints 'Worker v1.4.0' under Competitors. If it says 'Worker version unknown -- older than v1.4.0', the OLD Worker is still deployed. Keep in step with MARKET_RADAR_VERSION_HISTORY.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>Client version (browser console)</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>1.4.0</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="n"/>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>CLIENT_VERSION, market-radar.js</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>Press F12 on the page and look for '[Market Radar] script build' in the console. The HTML loads market-radar.js?v=2 so browsers fetch the new file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr">
+        <is>
+          <t>Geoapify free-plan licence (check before charging customers)</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>Free plan listed as 'Limited Commercial Use'; paid plans as 'Commercial Use'</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="n"/>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>External: geoapify.com/pricing -- checked 2026-09-20, not a code setting</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr">
+        <is>
+          <t>Read Geoapify's terms before selling a product that depends on this backstop. First paid tier listed: 'API 10', 10,000 credits/day, USD 59/month. Geoapify's Places docs say results may be cached/stored with no limits, so the 24h cache is fine.</t>
         </is>
       </c>
     </row>
@@ -1796,7 +1942,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -1839,6 +1985,13 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-20 CORRECTION (v1.4.0): on the settings tab, row 5 (Geoapify backstop key) used to name the WRONG secret -- GOOGLE_PLACES_API_KEY -- instead of GEOAPIFY_API_KEY. If you created a Worker secret from that name: (1) delete it, (2) create a secret named exactly GEOAPIFY_API_KEY, and (3) rotate the Geoapify key at myprojects.geoapify.com, because under the wrong name the key was sent to Google's servers on each analysis (where Google rejects it). Also added: the 'GEOAPIFY BACKSTOP &amp; DIAGNOSTICS' section at the bottom of the settings tab.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>